<commit_message>
B&N rev9 WIP: RFI-51 fixes (BE-47, BE-52), README/PARA_REVISAR draft
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev9.xlsx
+++ b/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev9.xlsx
@@ -1423,7 +1423,7 @@
     <t xml:space="preserve">RFI-01</t>
   </si>
   <si>
-    <t xml:space="preserve">CLOSED - estimator decision 2026-10-24 (rev1): perimeter walls types 1 / 1A / 1B / 1C are EXISTING (1/DM-101 legend solid = to remain + key note 3 "EXTERIOR WALL PATCH AND REPAIR AS REQUIRED TO MAINTAIN EXISTING FIRE RATING"; A-101 Construction Legend "EXISTING EXTERIOR WALL" / "EXISTING PARTITION"; A-002 "PERIMETER STUDS, INSULATION, VAPOR BARRIER F/I BY LL"). Perimeter framing (studs, track, bracing, 1B sheathing) EXCLUDED. Interior face patch &amp; repair (1/DM-101 key note 3, A-101 C5) = ALLOWANCE, amount: $ ________ (blank, estimator to fill). rev2 (estimator decision 2026-10-25): break room kitchenette W.R. on existing EXT-07 (6/A-412, 7/A-412) is INSIDE this patch &amp; repair allowance; allowance amount stays BLANK (decided).(rev7): A-410 types 1, 1A, 1B, 1C label the interior board "5/8" GYP BD BY FUTURE TENANT": EXCLUDED with that citation, consistent with this decision. A-413 7/8A general note "IF SHELVING IS TO BE INSTALLED ON EXISTING WALL, G.C. IS TO REMOVE AND REPLACE GYP. BOARD AS REQUIRED FOR INSTALLATION OF WOOD BLOCKING": inside this patch &amp; repair allowance.</t>
+    <t xml:space="preserve">CLOSED - estimator decision 2026-10-24 (rev1): perimeter walls types 1 / 1A / 1B / 1C are EXISTING (1/DM-101 legend solid = to remain + key note 3 "EXTERIOR WALL PATCH AND REPAIR AS REQUIRED TO MAINTAIN EXISTING FIRE RATING"; A-101 Construction Legend "EXISTING EXTERIOR WALL" / "EXISTING PARTITION"; A-002 "PERIMETER STUDS, INSULATION, VAPOR BARRIER F/I BY LL"). Perimeter framing (studs, track, bracing, 1B sheathing) EXCLUDED. Interior face patch &amp; repair (1/DM-101 key note 3, A-101 C5) = ALLOWANCE, amount: $ ________ (blank, estimator to fill). rev2 (estimator decision 2026-10-25): break room kitchenette W.R. on existing EXT-07 (6/A-412, 7/A-412) is INSIDE this patch &amp; repair allowance; allowance amount stays BLANK (decided). A-410 types 1, 1A, 1B, 1C label the interior board "5/8" GYP BD BY FUTURE TENANT": EXCLUDED with that citation, consistent with this decision. A-413 7/8A general note "IF SHELVING IS TO BE INSTALLED ON EXISTING WALL, G.C. IS TO REMOVE AND REPLACE GYP. BOARD AS REQUIRED FOR INSTALLATION OF WOOD BLOCKING": inside this patch &amp; repair allowance.</t>
   </si>
   <si>
     <t xml:space="preserve">Applied: - 417.43 LF of perimeter walls (17 walls); 3-5/8" stud 16,812.96 -&gt; 10,120.39 LF; 8" stud 2,332.99 -&gt; 0; 1/2" exterior sheathing 2,469.22 -&gt; 0 SF; bottom / top track 1,051.87 -&gt; 634.44 LF each; bracing 5,230.74 -&gt; 2,827.81 LF. Allowance: blank.; board by future tenant on the existing perimeter (A-410 types 1 / 1A / 1B / 1C): upper bound 417.43 LF x 25.0 = 10,436 SF 5/8" Type X if it were ever in our scope.</t>
@@ -1441,7 +1441,7 @@
     <t xml:space="preserve">RFI-03</t>
   </si>
   <si>
-    <t xml:space="preserve">B.O. deck is V.I.F. and sloped: 24'-0" (2/A-400B) to 25'-7" (2/A-400A); walls to deck loaded at 25'-0" (1/A-400A, 1/A-400B), east facade 25'-7", west 24'-0".(rev7): the elevations also print 21'-9" V.I.F. at the right end of 2/A-400A and 23'-8" V.I.F. on A-400B (joists sloping): the B.O. deck range is wider than 24'-0" to 25'-7".</t>
+    <t xml:space="preserve">B.O. deck is V.I.F. and sloped: 24'-0" (2/A-400B) to 25'-7" (2/A-400A); walls to deck loaded at 25'-0" (1/A-400A, 1/A-400B), east facade 25'-7", west 24'-0". the elevations also print 21'-9" V.I.F. at the right end of 2/A-400A and 23'-8" V.I.F. on A-400B (joists sloping): the B.O. deck range is wider than 24'-0" to 25'-7".</t>
   </si>
   <si>
     <t xml:space="preserve">Each 1 ft of deck height = 414.54 LF of studs-to-deck walls x 1 ft (studs, board where to deck, bracing rows)</t>
@@ -1450,7 +1450,7 @@
     <t xml:space="preserve">RFI-04</t>
   </si>
   <si>
-    <t xml:space="preserve">CLOSED - Review Item rev3 (estimator decision 2026-10-26): type 2 &gt; 22 ft: 3-5/8" 14 ga SJ + diagonal braces @ 32" O.C. to structure (3/A-410 Top Track Detail "PROVIDE DIAGONAL BRACING AT 32" O.C. TO STRUCTURE ABOVE (TYP.)"); brace member / length not printed - estimator choice 3-5/8" 20 ga stud x 4 ft at 45 deg.(rev7): same precedent applied to the Cafe 3-5/8" walls to deck (C-H2a, C-H2b, C-F): 14 ga SJ + 11 diagonal braces = 44.0 LF.</t>
+    <t xml:space="preserve">CLOSED - Review Item rev3 (estimator decision 2026-10-26): type 2 &gt; 22 ft: 3-5/8" 14 ga SJ + diagonal braces @ 32" O.C. to structure (3/A-410 Top Track Detail "PROVIDE DIAGONAL BRACING AT 32" O.C. TO STRUCTURE ABOVE (TYP.)"); brace member / length not printed - estimator choice 3-5/8" 20 ga stud x 4 ft at 45 deg. same precedent applied to the Cafe 3-5/8" walls to deck (C-H2a, C-H2b, C-F): 14 ga SJ + 11 diagonal braces = 44.0 LF.</t>
   </si>
   <si>
     <t xml:space="preserve">Applied: 117 braces x 4.0 ft = 468.0 LF (type 2) + 44.0 LF (Cafe) 3-5/8" 20 ga stud (member and length = estimator choice). Citation history: rev0-rev2 cited the partition type 3 section, rev3-rev6 cited 8/A-410 (that bubble is the Typ. Connection Detail); the Top Track Detail is bubble 3/A-410.</t>
@@ -1816,7 +1816,7 @@
     <t xml:space="preserve">RFI-46</t>
   </si>
   <si>
-    <t xml:space="preserve">F/A-221 "3 5/8" METAL STUDS @ 16" O.C. TO BOTTOM OF NESTED STUD BRACING": the nested stud bracing member is not drawn; studs carried to deck (estimator decision RI 7).(rev8): the same phrase is printed on the partition types 3 and 4 (3/A-410, 4/A-410): nested stud at the top of each wall.</t>
+    <t xml:space="preserve">F/A-221 "3 5/8" METAL STUDS @ 16" O.C. TO BOTTOM OF NESTED STUD BRACING": the nested stud bracing member is not drawn; studs carried to deck (estimator decision RI 7). the same phrase is printed on the partition types 3 and 4 (3/A-410, 4/A-410): nested stud at the top of each wall.</t>
   </si>
   <si>
     <t xml:space="preserve">Carried 6.52 LF (F) + 122.32 LF (types 3 / 4) 3-5/8" stud; define member / elevation; if not required: minus both.</t>
@@ -1870,7 +1870,7 @@
     <t xml:space="preserve">RFI-53</t>
   </si>
   <si>
-    <t xml:space="preserve">Light fixtures in the Cafe GWB bands (11'-6" and 9'-0", 1/A-121): fixture count in the bands not taken; 5/A-121 "PROVIDE ADDITIONAL WIRE SUPPORT AT ALL LIGHT FIXTURES".(rev8): E-301 Sec. 265119: "THIS CONTRACTOR SHALL PROVIDE AND INSTALL ALL NECESSARY SUPPORT MEDIA FOR ALL LIGHTING FIXTURES ... FIXTURES SHALL NOT BE SUPPORTED FROM ROOF DECK" - overlap with the 5/A-121 fixture wires carried.</t>
+    <t xml:space="preserve">Light fixtures in the Cafe GWB bands (11'-6" and 9'-0", 1/A-121): fixture count in the bands not taken; 5/A-121 "PROVIDE ADDITIONAL WIRE SUPPORT AT ALL LIGHT FIXTURES". E-301 Sec. 265119: "THIS CONTRACTOR SHALL PROVIDE AND INSTALL ALL NECESSARY SUPPORT MEDIA FOR ALL LIGHTING FIXTURES ... FIXTURES SHALL NOT BE SUPPORTED FROM ROOF DECK" - overlap with the 5/A-121 fixture wires carried.</t>
   </si>
   <si>
     <t xml:space="preserve">Each fixture in a band = + 1 hanger x 13.5 / 16.0 ft wire. If the fixture supports are by the electrical contractor (E-301 265119): - 401.0 LF hanger wire (29 hangers).</t>
@@ -1882,7 +1882,7 @@
     <t xml:space="preserve">Fastener counts not printed: 7/A-210 3"x3"x16 ga clip angles (count per header end); cement board screw spacing (manufacturer standard 8" O.C. used); plywood screws per A-410 note 8.D (24" field / 12" perimeter on 4x8 sheets).</t>
   </si>
   <si>
-    <t xml:space="preserve">Carried: clip angles 7/A-210 4 pcs; cement board screws 1686 pcs; plywood screws 2331 pcs - adjust to the estimator yields. Framing screws count the stud pieces of the walls and column wraps (781) by gauge (A-410 note 8.A); the 8/A-410 #8 screws (top chord, cross members, track) have their own row; the other detail members (braces, bracing clips) are in the Tek screw row. 9/A-410 calls #8 screws stud to track while note 8.A calls #10-16 on 18/16 ga - carried per 8.A.(rev8): relief channel to structure carried with 8/A-410 #8 pan head screws (291 pcs) + P.A.F. at cross members (282 pcs); note 8.C X-EDNI (2 rows @ 16" = 720 pcs) is the alternative if the track bears directly on structural steel. Slab pins carried per note 8.F (2 rows @ 16" X-DNI); 9/A-410 alternative 0.177" PAF @ 24" = - 640.61 pcs. 8/A-210 "(8) #10-16 TEKS 16"O.C., TYP." read as 8 per station at 16" O.C. (520 pcs carried); if 8 per member in total: - 464 pcs. 7/A-210 head attachment clips: 2 assumed (16 screws), count not printed.</t>
+    <t xml:space="preserve">Carried: clip angles 7/A-210 4 pcs; cement board screws 1686 pcs; plywood screws 2331 pcs - adjust to the estimator yields. Framing screws count the stud pieces of the walls and column wraps (781) by gauge (A-410 note 8.A); the 8/A-410 #8 screws (top chord, cross members, track) have their own row; 5/A-410 bracing clips are in the Tek screw row; diagonal brace end screws (3/A-410) are not printed and not carried (if 2 per end: + 512 #8). 9/A-410 calls #8 screws stud to track while note 8.A calls #10-16 on 18/16 ga - carried per 8.A. relief channel to structure carried with 8/A-410 #8 pan head screws (291 pcs) + P.A.F. at cross members (282 pcs); note 8.C X-EDNI (2 rows @ 16" = 720 pcs) is the alternative if the track bears directly on structural steel. Slab pins carried per note 8.F (2 rows @ 16" X-DNI); 9/A-410 alternative 0.177" PAF @ 24" = - 518.29 pcs (518.29 LF of interior bottom track on slab). 8/A-210 "(8) #10-16 TEKS 16"O.C., TYP." read as 8 per station at 16" O.C. (520 pcs carried); if 8 per member in total: - 464 pcs. 7/A-210 head attachment clips: 2 assumed (16 screws), count not printed.</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-54</t>

</xml_diff>